<commit_message>
Complete 퇴직급여충당부채 sheet from Severance working paper (H2/H2-1)
Fill the retirement benefit obligation estimate from the Severance
working paper: DB lump-sum measurement under K-GAAP, 50 covered
employees, recomputed 추계액 (2,338,962,958 vs company 2,341,038,944,
CTT immaterial pass), pension plan asset reconciliation (하나은행
2,486,524,515), and reclassification of the 145,485,571 excess to
기타투자자산. Inherent risk assessed Standard (low uncertainty/
complexity/subjectivity).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WBECbymcckWM3Hc9PV367F
</commit_message>
<xml_diff>
--- a/MAM_Tool_ISA540R_Accounting_estimates_PAT_2026YE.xlsx
+++ b/MAM_Tool_ISA540R_Accounting_estimates_PAT_2026YE.xlsx
@@ -28057,7 +28057,7 @@
       </c>
       <c r="L1" s="373" t="inlineStr">
         <is>
-          <t>(첨부6 예정)</t>
+          <t>H2 / H2-1</t>
         </is>
       </c>
       <c r="M1" s="374" t="n"/>
@@ -28099,7 +28099,11 @@
           <t>Prepared by:</t>
         </is>
       </c>
-      <c r="L2" s="376" t="inlineStr"/>
+      <c r="L2" s="376" t="inlineStr">
+        <is>
+          <t>HSH</t>
+        </is>
+      </c>
       <c r="M2" s="374" t="n"/>
       <c r="N2" s="374" t="n"/>
       <c r="O2" s="43" t="n"/>
@@ -28131,7 +28135,11 @@
           <t>Date:</t>
         </is>
       </c>
-      <c r="L3" s="375" t="inlineStr"/>
+      <c r="L3" s="375" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
       <c r="M3" s="374" t="n"/>
       <c r="N3" s="374" t="n"/>
       <c r="O3" s="43" t="n"/>
@@ -28167,7 +28175,11 @@
           <t>Reviewed by:</t>
         </is>
       </c>
-      <c r="L4" s="376" t="inlineStr"/>
+      <c r="L4" s="376" t="inlineStr">
+        <is>
+          <t>LJM</t>
+        </is>
+      </c>
       <c r="M4" s="374" t="n"/>
       <c r="N4" s="374" t="n"/>
       <c r="O4" s="43" t="n"/>
@@ -28251,8 +28263,7 @@
       <c r="B7" s="378" t="inlineStr">
         <is>
           <t>SCOTABD: 퇴직급여충당부채  /  관련 주장(Assertion): 평가(Valuation) 및 완전성(Completeness)
-WCGW: 퇴직급여충당부채가 회계기준에 따라 완전하고 정확하게 계상되지 않을 수 있음.
-※ 세부 내용은 조서(첨부6) 입수 후 확정 예정.</t>
+WCGW: 재직 임직원에 대한 퇴직급여충당부채가 완전하고 정확하게 계상되지 않을 수 있음.</t>
         </is>
       </c>
       <c r="C7" s="43" t="n"/>
@@ -28389,8 +28400,7 @@
       <c r="A13" s="55" t="n"/>
       <c r="B13" s="379" t="inlineStr">
         <is>
-          <t>회사는 종업원에 대한 퇴직급여제도를 운영하며 이에 따라 퇴직급여충당부채를 인식함. 이연법인세 조서(첨부4) 상 당기말 퇴직급여충당부채 관련 일시적차이는 2,341,038,944원이며 동액의 퇴직연금(사외적립자산)이 대응됨.
-※ 조서(첨부6) 입수 후 작성 예정 (Pending receipt of working paper).</t>
+          <t>회사는 확정급여형(DB) 퇴직급여제도를 운영하며, 재직 임직원에 대해 보고기간말 현재 전 임직원이 일시에 퇴직할 경우 지급하여야 할 퇴직금 추계액을 퇴직급여충당부채로 인식함. 당기말 퇴직급여충당부채는 2,341,038,944원(기초 2,095,898,236 + 설정 413,112,884 - 지급 167,972,176)이며, 퇴직연금운용자산(퇴직보험예치금)은 하나은행에 예치되어 기말 2,486,524,515원임. 당기 중 제도의 중요한 변경은 없음.</t>
         </is>
       </c>
       <c r="C13" s="374" t="n"/>
@@ -28492,8 +28502,7 @@
       <c r="A17" s="55" t="n"/>
       <c r="B17" s="382" t="inlineStr">
         <is>
-          <t>적용 재무보고체계는 일반기업회계기준(K-GAAP)임. 퇴직급여충당부채는 보고기간말 현재 전 임직원이 일시에 퇴직할 경우 지급하여야 할 퇴직금 추계액을 기준으로 인식함(회사 부담분).
-※ 조서(첨부6) 입수 후 작성 예정 (Pending receipt of working paper).</t>
+          <t>적용 재무보고체계는 일반기업회계기준(K-GAAP)임. 퇴직급여충당부채는 보고기간말 현재 전 임직원이 일시에 퇴직할 경우 지급하여야 할 퇴직금 추계액으로 인식하며, 근로자퇴직급여보장법 및 회사 퇴직금 지급규정에 따라 산정함. 퇴직연금운용자산은 공정가치로 측정함.</t>
         </is>
       </c>
       <c r="C17" s="374" t="n"/>
@@ -28605,7 +28614,7 @@
       <c r="A21" s="55" t="n"/>
       <c r="B21" s="382" t="inlineStr">
         <is>
-          <t>근로자퇴직급여보장법 등 관련 법규를 고려함. 세부 규제요인은 조서(첨부6) 입수 후 확정 예정.</t>
+          <t>근로자퇴직급여보장법 및 관련 세법상 퇴직급여 손금규정을 고려함. 그 외 추정에 영향을 미치는 특별한 규제요인은 식별되지 않음.</t>
         </is>
       </c>
       <c r="C21" s="374" t="n"/>
@@ -28763,8 +28772,7 @@
     <row r="27" customFormat="1" s="65">
       <c r="B27" s="382" t="inlineStr">
         <is>
-          <t>퇴직급여충당부채는 재무제표에 중요하고 급여·근속연수 등 데이터에 기초한 추정을 수반하므로 중요왜곡표시위험이 존재함(잠정 판단).
-※ 조서(첨부6) 입수 후 작성 예정 (Pending receipt of working paper).</t>
+          <t>퇴직급여충당부채가 재무제표에 중요하고(2,341백만원) 임직원별 급여·근속연수 데이터에 기초한 추정을 수반하므로 표준수준(Standard)의 중요왜곡표시위험이 존재함. 다만 K-GAAP상 일시퇴직 기준 추계로 장기 보험수리적 가정이 개입하지 않아 추정불확실성이 낮음.</t>
         </is>
       </c>
       <c r="C27" s="374" t="n"/>
@@ -28988,7 +28996,7 @@
       <c r="A36" s="55" t="n"/>
       <c r="B36" s="382" t="inlineStr">
         <is>
-          <t>재무팀 및 본사(VF)의 검토·보고체계를 통해 퇴직급여 관련 회계처리가 감독됨. 세부 내용은 조서(첨부6) 입수 후 확정 예정.</t>
+          <t>재무팀이 퇴직급여충당부채 추계 및 퇴직연금 운용현황을 관리하고, 본사(VF) 보고체계를 통해 관련 회계처리가 감독됨. 퇴직연금은 금융기관(하나은행) 운용현황보고서 및 조회서로 검증됨.</t>
         </is>
       </c>
       <c r="C36" s="374" t="n"/>
@@ -29100,7 +29108,7 @@
       <c r="A40" s="55" t="n"/>
       <c r="B40" s="382" t="inlineStr">
         <is>
-          <t>회사는 임직원 현황 및 급여·근속연수 데이터를 관리하여 퇴직급여충당부채 추계액을 산정함. 세부 내용은 조서(첨부6) 입수 후 확정 예정.</t>
+          <t>회사는 재직 임직원 현황 및 급여·근속연수 데이터를 인사·급여시스템으로 관리하여 퇴직금 추계액을 산정하고, 퇴직연금 적립현황을 모니터링함. 퇴직자 발생 시 퇴직금 정산·지급을 처리함.</t>
         </is>
       </c>
       <c r="C40" s="374" t="n"/>
@@ -29237,7 +29245,7 @@
       <c r="A45" s="55" t="n"/>
       <c r="B45" s="382" t="inlineStr">
         <is>
-          <t>① 퇴직금 추계액 명세의 작성 및 검토, ② 퇴직연금(사외적립자산) 대사, ③ 회계처리의 검토·승인. 세부 통제는 조서(첨부6) 입수 후 확정 예정.</t>
+          <t>① 급여대장 기준 추계대상 인원의 식별 및 검토, ② 임직원별 퇴직금 추계액 계산의 검토·승인, ③ 퇴직연금 운용현황보고서·금융기관 조회서 대사, ④ 퇴직금 지급 시 원천징수·지출결의·이체 확인. (식별된 통제는 Atlas의 해당 노드에 반영 필요.)</t>
         </is>
       </c>
       <c r="C45" s="374" t="n"/>
@@ -29365,7 +29373,7 @@
     <row r="51" customFormat="1" s="55">
       <c r="B51" s="382" t="inlineStr">
         <is>
-          <t>인사·급여 시스템의 임직원별 급여·근속연수 데이터를 근거로 퇴직금 추계액을 산출하여 총계정원장·재무제표에 반영함. 세부 내용은 조서(첨부6) 입수 후 확정 예정.</t>
+          <t>인사·급여시스템의 임직원별 급여(최근 3개월)·상여·입사일 데이터를 근거로 평균임금 및 근속일수를 산출하고, 이를 곱하여 임직원별 퇴직금 추계액을 산정한 뒤 합산하여 퇴직급여충당부채로 총계정원장·재무제표에 반영함.</t>
         </is>
       </c>
       <c r="C51" s="374" t="n"/>
@@ -29489,8 +29497,7 @@
     <row r="55" customFormat="1" s="55">
       <c r="B55" s="382" t="inlineStr">
         <is>
-          <t>[방법] 보고기간말 기준 전 임직원 일시퇴직 가정에 따른 퇴직금 추계액을 퇴직급여충당부채로 인식(K-GAAP). 세부 방법은 조서(첨부6) 입수 후 확정 예정.
-※ 조서(첨부6) 입수 후 작성 예정 (Pending receipt of working paper).</t>
+          <t>[방법] 임직원별 평균임금(최근 3개월 급여 + 산정상여, 연간상여의 3/12 반영) 기준 일별 평균임금 × 근속일수로 퇴직금 추계액을 산정하고, 전 임직원 합계를 퇴직급여충당부채로 인식함(K-GAAP 일시퇴직 기준). 육아휴직자는 연봉테이블상 연봉으로 산정함. 전기와 동일한 방법을 계속 적용하고 있으며 계속 적용이 적정한 것으로 판단됨.</t>
         </is>
       </c>
       <c r="C55" s="374" t="n"/>
@@ -29614,7 +29621,7 @@
     <row r="59" customFormat="1" s="55">
       <c r="B59" s="382" t="inlineStr">
         <is>
-          <t>주요 가정은 급여수준, 근속연수 및 퇴직금 지급률 등임. 보험수리적 가정 적용 여부 등 세부 사항은 조서(첨부6) 입수 후 확정 예정.</t>
+          <t>주요 가정은 ① 보고기간말 전 임직원 일시퇴직 가정, ② 평균임금 산정기준(최근 3개월 급여 및 연간 상여의 3/12 반영)임. K-GAAP상 할인율·이직률·사망률·임금상승률 등 장기 보험수리적 가정은 적용하지 않음.</t>
         </is>
       </c>
       <c r="C59" s="374" t="n"/>
@@ -29740,7 +29747,7 @@
       <c r="A63" s="65" t="n"/>
       <c r="B63" s="382" t="inlineStr">
         <is>
-          <t>사용 데이터는 임직원별 급여·근속연수 및 퇴직금 지급규정임. 세부 데이터 검증은 조서(첨부6) 입수 후 확정 예정.</t>
+          <t>사용 데이터는 급여대장(총지급액-연차수당), 상여내역, 임직원별 입사일·근속일수 및 퇴직연금 운용현황보고서임. 급여대장 58명 중 1년 미만 입사자 8명·퇴사자 0명을 제외한 추계대상 50명이 회사 계산인원과 일치함(차이 0).</t>
         </is>
       </c>
       <c r="C63" s="374" t="n"/>
@@ -29868,7 +29875,7 @@
       <c r="A67" s="65" t="n"/>
       <c r="B67" s="382" t="inlineStr">
         <is>
-          <t>경영진의 추정불확실성 평가 내용은 조서(첨부6) 입수 후 확정 예정.</t>
+          <t>K-GAAP상 일시퇴직 기준 추계로 추정불확실성이 낮음. 회사는 실제 급여·근속연수 데이터에 근거하여 추계액을 산정하며 별도의 민감도분석은 수행하지 않음. 퇴직연금운용자산은 금융기관 평가액(공정가치)으로 측정함.</t>
         </is>
       </c>
       <c r="C67" s="374" t="n"/>
@@ -29996,7 +30003,7 @@
       <c r="A71" s="65" t="n"/>
       <c r="B71" s="382" t="inlineStr">
         <is>
-          <t>전기 퇴직급여충당부채의 당기 변동(설정·지급) 및 추정의 적정성은 조서(첨부6) 입수 후 검토 예정.</t>
+          <t>전기 퇴직급여충당부채 2,095,898,236원의 당기 변동(설정 413,112,884, 지급 167,972,176)을 검토함. 당기 퇴직자 2명에 대한 퇴직금 지급액을 퇴직소득원천징수영수증·이체증으로 확인함. 충당금전입액(413,112,884)과 PL 퇴직급여의 차이(3,380,976원, 직영점 기간제 근로자 관련)는 CTT 미만으로 확인되었으며, 경영진 편의의 징후는 없음.</t>
         </is>
       </c>
       <c r="C71" s="374" t="n"/>
@@ -30124,7 +30131,7 @@
       <c r="A75" s="65" t="n"/>
       <c r="B75" s="382" t="inlineStr">
         <is>
-          <t>경영진의 전문가(보험계리인 등) 이용 여부는 조서(첨부6) 입수 후 확정 예정.</t>
+          <t>K-GAAP상 일시퇴직 추계로 보험계리인 등 경영진의 전문가는 이용되지 않음.</t>
         </is>
       </c>
       <c r="C75" s="374" t="n"/>
@@ -30430,7 +30437,7 @@
       <c r="A85" s="65" t="n"/>
       <c r="B85" s="382" t="inlineStr">
         <is>
-          <t>감사팀 스킬 및 지식의 적정성은 조서(첨부6) 입수 후 확정 예정.</t>
+          <t>퇴직금 추계액 재계산 및 퇴직연금 대사는 감사팀의 통상적 감사기술로 충분하며 별도의 전문 스킬은 요구되지 않음.</t>
         </is>
       </c>
       <c r="C85" s="374" t="n"/>
@@ -30936,7 +30943,7 @@
       <c r="A104" s="65" t="n"/>
       <c r="B104" s="382" t="inlineStr">
         <is>
-          <t>K-GAAP상 일시퇴직 기준 추계액으로 산정 시 추정불확실성은 낮은 편으로 잠정 판단함. ※ 조서(첨부6) 입수 후 작성 예정 (Pending receipt of working paper).</t>
+          <t>K-GAAP상 보고기간말 일시퇴직 기준 추계로 장기 보험수리적 가정이 개입하지 않아 측정의 추정불확실성이 낮음.</t>
         </is>
       </c>
       <c r="C104" s="374" t="n"/>
@@ -31145,7 +31152,7 @@
       <c r="A111" s="65" t="n"/>
       <c r="B111" s="382" t="inlineStr">
         <is>
-          <t>급여·근속연수 데이터에 기초한 추계로 복잡성은 낮은 편으로 잠정 판단함. ※ 조서(첨부6) 입수 후 작성 예정 (Pending receipt of working paper).</t>
+          <t>임직원별 평균임금 × 근속일수의 정형화된 계산으로 복잡한 모델이 개입하지 않아 복잡성이 낮음.</t>
         </is>
       </c>
       <c r="C111" s="374" t="n"/>
@@ -31293,7 +31300,7 @@
     <row r="116" ht="15" customFormat="1" customHeight="1" s="65">
       <c r="B116" s="382" t="inlineStr">
         <is>
-          <t>일시퇴직 기준 추계액으로 판단개입 여지가 제한적이어서 주관성은 낮은 편으로 잠정 판단함. ※ 조서(첨부6) 입수 후 작성 예정 (Pending receipt of working paper).</t>
+          <t>추계기준이 K-GAAP 및 지급규정으로 정해져 있어 판단개입 여지가 제한적이므로 주관성이 낮음.</t>
         </is>
       </c>
       <c r="C116" s="374" t="n"/>
@@ -31490,7 +31497,7 @@
     <row r="123" ht="15" customFormat="1" customHeight="1" s="65">
       <c r="B123" s="382" t="inlineStr">
         <is>
-          <t>기타 고유위험요인은 조서(첨부6) 입수 후 확정 예정.</t>
+          <t>퇴직연금운용자산이 퇴직급여충당부채를 초과하여 초과분(145,485,571원)을 기타투자자산으로 재분류하는 회계처리(수정사항 제시)를 검토함. 경영진 편의의 징후는 없음.</t>
         </is>
       </c>
       <c r="C123" s="374" t="n"/>
@@ -31605,8 +31612,7 @@
     <row r="128" ht="15" customFormat="1" customHeight="1" s="65">
       <c r="B128" s="387" t="inlineStr">
         <is>
-          <t>잠정적으로 고유위험을 표준(Standard)으로 선택함. 최종 평가는 조서(첨부6) 입수 후 확정 예정.
-※ 조서(첨부6) 입수 후 작성 예정 (Pending receipt of working paper).</t>
+          <t>일시퇴직 기준 추계로 추정불확실성·복잡성·주관성이 모두 낮으므로 고유위험을 표준(Standard)으로 선택함(계산된 제안 수준과 동일).</t>
         </is>
       </c>
       <c r="C128" s="374" t="n"/>
@@ -32014,7 +32020,7 @@
     <row r="144" ht="15" customFormat="1" customHeight="1" s="65">
       <c r="B144" s="387" t="inlineStr">
         <is>
-          <t>실증절차(퇴직금 추계액 재계산 및 사외적립자산 대사) 중심으로 계획함(잠정). 세부 내용은 조서(첨부6) 입수 후 확정 예정.</t>
+          <t>퇴직금 추계액 재계산, 인원 완전성 검토 및 퇴직연금 외부조회 등 실증절차만으로 충분하고 적합한 감사증거를 확보할 수 있어 통제 운영효과성에 의존하지 않음.</t>
         </is>
       </c>
       <c r="C144" s="374" t="n"/>
@@ -32476,8 +32482,7 @@
       <c r="B161" s="382" t="inlineStr">
         <is>
           <t>[접근법: 경영진이 추정치를 산출한 방법의 검토 - ISA 540.22~27]
-퇴직금 추계액 재계산, 퇴직연금(사외적립자산) 대사, 관련 회계처리 및 주석 검토를 수행할 예정임.
-※ 조서(첨부6) 입수 후 작성 예정 (Pending receipt of working paper).</t>
+① 명세서 대사: 회사 계산내역과 BS상 퇴직급여충당부채(2,341,038,944원)·퇴직보험예치금(2,486,524,515원)이 일치함을 확인함. ② 인원 완전성 검토: 급여대장(58명)에서 1년 미만 입사자(8명)·퇴사자(0명)를 제외한 추계대상 50명이 회사 계산인원과 일치함(차이 0). ③ 재계산 검증: 임직원별 평균임금·근속일수 기준 추계액을 재계산함(회사 2,341,038,944원 대 감사인 2,338,962,958원, 차이 -2,075,986원은 CTT 미만 Immaterial pass). ④ 퇴직연금 검증: 운용현황보고서 및 금융기관(하나은행) 조회서로 기말 적립금(2,486,524,515원)을 대사함(차이 0). ⑤ 퇴직금 지급 검토: 당기 퇴직자 2명의 퇴직소득원천징수영수증·지출결의서·이체증을 확인함. ⑥ 계정분류: 퇴직연금이 충당부채를 초과하는 145,485,571원을 기타투자자산으로 재분류하는 수정사항을 제시함. 결론: 상기 수정사항(초과분 재분류)을 제외하고 중요성 관점에서 적정함.</t>
         </is>
       </c>
       <c r="C161" s="374" t="n"/>
@@ -32690,7 +32695,7 @@
     <row r="170" customFormat="1" s="158">
       <c r="B170" s="390" t="inlineStr">
         <is>
-          <t>(첨부6 조서 입수 후 기재 예정)</t>
+          <t>H2(Lead), H2-1(퇴직급여추계액 재계산), H2-2(연차유급휴가)</t>
         </is>
       </c>
       <c r="C170" s="243" t="n"/>
@@ -32718,7 +32723,7 @@
     <row r="171" ht="15.75" customFormat="1" customHeight="1" s="65" thickBot="1">
       <c r="B171" s="391" t="inlineStr">
         <is>
-          <t>※ 조서(첨부6) 입수 후 작성 예정 (Pending receipt of working paper).</t>
+          <t>상기 절차는 퇴직급여 감사조서(Lead H2, 재계산 H2-1)에 문서화되어 있으며, 초과분 재분류 수정사항 반영 후 중요성 관점에서 적정함.</t>
         </is>
       </c>
       <c r="C171" s="244" t="n"/>
@@ -32882,7 +32887,7 @@
     <row r="177" ht="15" customFormat="1" customHeight="1" s="65">
       <c r="B177" s="379" t="inlineStr">
         <is>
-          <t>세부 내용은 조서(첨부6) 입수 후 확정 예정.</t>
+          <t>표준위험 수준에 상응하는 전문가적 회의주의를 적용함. 추계대상 인원의 완전성 및 평균임금 산정기준의 적정성을 비판적으로 검토함.</t>
         </is>
       </c>
       <c r="C177" s="374" t="n"/>
@@ -32990,7 +32995,7 @@
     <row r="181" ht="15" customFormat="1" customHeight="1" s="65">
       <c r="B181" s="379" t="inlineStr">
         <is>
-          <t>세부 내용은 조서(첨부6) 입수 후 확정 예정.</t>
+          <t>인원 완전성 검토 및 임직원별 추계액 재계산을 중심으로 실증절차를 수행하고, 퇴직연금은 외부 조회로 검증함.</t>
         </is>
       </c>
       <c r="C181" s="374" t="n"/>
@@ -33098,7 +33103,7 @@
     <row r="185" ht="15" customFormat="1" customHeight="1" s="65">
       <c r="B185" s="379" t="inlineStr">
         <is>
-          <t>세부 내용은 조서(첨부6) 입수 후 확정 예정.</t>
+          <t>표준위험 수준으로 통상적 감사팀 구성으로 충분하며 별도의 추가 자원은 필요하지 않음.</t>
         </is>
       </c>
       <c r="C185" s="374" t="n"/>
@@ -33191,7 +33196,7 @@
     <row r="189" ht="15" customFormat="1" customHeight="1" s="65">
       <c r="B189" s="395" t="inlineStr">
         <is>
-          <t>세부 내용은 조서(첨부6) 입수 후 확정 예정.</t>
+          <t>표준위험 수준에 상응하는 통상적 검토·감독을 수행함.</t>
         </is>
       </c>
       <c r="C189" s="374" t="n"/>

</xml_diff>